<commit_message>
Daily job digest update (2026-08-23)
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -1,15 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Job Digest" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Job Digest" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Digest'!$A$1:$J$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -494,6 +496,12 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J1"/>
+  <dataValidations count="1">
+    <dataValidation sqref="J2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"No,Applied,Interviewing,Rejected,Not Interested"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Daily job digest update (2026-09-05)
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job Digest" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Digest'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job Digest'!$A$1:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +31,10 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -58,10 +62,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -428,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -495,10 +502,160 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>docker, ci/cd, kubernetes, prometheus, grafana, linux</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Infrastructure &amp;amp; Platform Engineer (Junior–Mid Level)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>See listing</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Cairo/Giza area</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Thu, 06 Aug 2026 17:24:23 GMT</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Wuzzuf</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>https://wuzzuf.net/jobs/p/153c31da-ea8d-4709-ba54-1961c666665f-Infrastructure---Platform-Engineer-Junior–Mid-Level-WITHIN-EARTH-HOLIDAYS-Giza-Egypt</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>aws, docker, ci/cd, git, jenkins, react</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>DevOps Engineer</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>See listing</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Cairo/Giza area</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Wed, 08 Jul 2026 16:41:06 GMT</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Wuzzuf</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>https://wuzzuf.net/jobs/p/75fd08e8-6be9-4821-88c7-d5827171c8e4-DevOps-Engineer-Bright-Creations-Giza-Egypt</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>linux</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Junior Site Reliability Engineer (SRE) L3</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>See listing</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Cairo/Giza area</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Mon, 24 Aug 2026 12:41:23 GMT</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Wuzzuf</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>https://wuzzuf.net/jobs/p/7c073f86-afc0-4c85-9dee-c0ef1bc6943c-Junior-Site-Reliability-Engineer-SRE-L3-Vertex-Technologies-Cairo-Egypt</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:J4"/>
   <dataValidations count="1">
-    <dataValidation sqref="J2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="J2:J4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"No,Applied,Interviewing,Rejected,Not Interested"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>